<commit_message>
fix(employees): redesign UI for consistency and fix missing API integration
- Rebuilt HTML with modern design system matching rest of app (dark theme, sidebar)
- Fixed DOM ID mismatches between HTML and JavaScript (modal, form fields, tabs)
- Updated tab structure for proper state management
- Split employee rendering into pending/completed tables
- Fixed JavaScript to work with new HTML structure
- Simplified form validation module
- Improved error handling for authentication failures
</commit_message>
<xml_diff>
--- a/exports/registros-IT.xlsx
+++ b/exports/registros-IT.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Fecha / Hora</t>
   </si>
@@ -94,7 +94,10 @@
     <t>alta</t>
   </si>
   <si>
-    <t>pendiente</t>
+    <t>completado</t>
+  </si>
+  <si>
+    <t>16/06/2026, 11:30:44</t>
   </si>
 </sst>
 </file>
@@ -120,7 +123,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -130,6 +133,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4F46E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF10B981"/>
       </patternFill>
     </fill>
     <fill>
@@ -170,10 +178,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -624,7 +632,7 @@
         <v>27</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>24</v>
@@ -644,6 +652,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>